<commit_message>
fix: update academic question bank, default mcq selection, excel category imports, and cq counts per passage
</commit_message>
<xml_diff>
--- a/public/cq-question-demo.xlsx
+++ b/public/cq-question-demo.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="22">
   <si>
     <t>Stimulus (উদ্দীপক)</t>
   </si>
@@ -47,6 +47,9 @@
     <t>Job Category (বিষয়)</t>
   </si>
   <si>
+    <t>Sub Category (অধ্যায়/গল্পের নাম)</t>
+  </si>
+  <si>
     <t>উদ্দীপক: ১৯৭১ সালের ২৬শে মার্চ বঙ্গবন্ধু শেখ মুজিবুর রহমান বাংলাদেশের স্বাধীনতা ঘোষণা করেন। দীর্ঘ নয় মাস রক্তক্ষয়ী যুদ্ধের পর ১৬ই ডিসেম্বর বাংলাদেশ বিজয় অর্জন করে।</t>
   </si>
   <si>
@@ -74,7 +77,10 @@
     <t>উক্তিটি যথার্থ কারণ দীর্ঘ নয় মাসের মুক্তিসংগ্রাম ও আত্মত্যাগের ইতিহাস স্মরণ করার মাধ্যমে নতুন প্রজন্মের মাঝে দেশপ্রেমের মূল্যবোধ সুদৃঢ় হয়।</t>
   </si>
   <si>
-    <t>ইতিহাস</t>
+    <t>বাংলা সাহিত্য</t>
+  </si>
+  <si>
+    <t>আম-আঁটির ভেঁপু</t>
   </si>
 </sst>
 </file>
@@ -414,7 +420,7 @@
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
   </sheetPr>
-  <dimension ref="A1:J2"/>
+  <dimension ref="A1:K2"/>
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col min="1" max="1" width="193.381" bestFit="true" customWidth="true" style="0"/>
@@ -427,9 +433,10 @@
     <col min="8" max="8" width="111.973" bestFit="true" customWidth="true" style="0"/>
     <col min="9" max="9" width="163.817" bestFit="true" customWidth="true" style="0"/>
     <col min="10" max="10" width="23.423" bestFit="true" customWidth="true" style="0"/>
+    <col min="11" max="11" width="38.848" bestFit="true" customWidth="true" style="0"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10">
+    <row r="1" spans="1:11">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -460,37 +467,43 @@
       <c r="J1" t="s">
         <v>9</v>
       </c>
+      <c r="K1" t="s">
+        <v>10</v>
+      </c>
     </row>
-    <row r="2" spans="1:10">
+    <row r="2" spans="1:11">
       <c r="A2" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B2" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C2" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D2" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="E2" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="F2" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="G2" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="H2" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="I2" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="J2" t="s">
-        <v>19</v>
+        <v>20</v>
+      </c>
+      <c r="K2" t="s">
+        <v>21</v>
       </c>
     </row>
   </sheetData>

</xml_diff>